<commit_message>
quad encoder distance calculation
</commit_message>
<xml_diff>
--- a/madi/301 speed data.xlsx
+++ b/madi/301 speed data.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madi/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madi/Desktop/COMPSYS301_team2/madi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1388AC9-565F-E44E-AFB5-9C449B36B35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6434248-AC0E-3649-BA0A-E8F6C8DA6138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" activeTab="1" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="cmo speed" sheetId="1" r:id="rId1"/>
+    <sheet name="quad encoder distance " sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>CMP Value</t>
   </si>
@@ -57,6 +58,27 @@
   </si>
   <si>
     <t>Speed (m/s)</t>
+  </si>
+  <si>
+    <t>Conditions:</t>
+  </si>
+  <si>
+    <t>Batteries were not fully charged</t>
+  </si>
+  <si>
+    <t>No line following so the robot was going quite curved - we were manually straightening</t>
+  </si>
+  <si>
+    <t>Quad encoder #</t>
+  </si>
+  <si>
+    <t>Distance</t>
+  </si>
+  <si>
+    <t>Avg Distance</t>
+  </si>
+  <si>
+    <t>Quad</t>
   </si>
 </sst>
 </file>
@@ -151,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -162,10 +184,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -174,9 +193,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -279,7 +311,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$G$2</c:f>
+              <c:f>'cmo speed'!$G$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -389,7 +421,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$3:$D$20</c:f>
+              <c:f>'cmo speed'!$D$3:$D$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
@@ -416,7 +448,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$G$3:$G$20</c:f>
+              <c:f>'cmo speed'!$G$3:$G$20</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="18"/>
@@ -536,7 +568,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -750,7 +782,614 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Distance</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> travelled vs quad encoder value</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="6.1681959176590521E-2"/>
+          <c:y val="2.9154507795769995E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'quad encoder distance '!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Avg Distance</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:forward val="250"/>
+            <c:backward val="250"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.15770346630224941"/>
+                  <c:y val="-0.12721083568220976"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="tx1">
+                            <a:lumMod val="65000"/>
+                            <a:lumOff val="35000"/>
+                          </a:schemeClr>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" baseline="0"/>
+                      <a:t>distance = 0.001(quad) + 0.0483</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US"/>
+                  </a:p>
+                </c:rich>
+              </c:tx>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'quad encoder distance '!$B$3:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>750</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'quad encoder distance '!$D$3:$D$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>0.27666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.54666666666666675</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.77833333333333332</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0033333333333332</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4E6C-C140-9A24-2C878967AADF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1248083968"/>
+        <c:axId val="1248096512"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1248083968"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Quad encoder value</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1248096512"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1248096512"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> travelled</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1248083968"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1306,6 +1945,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1327,6 +2482,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7C5DB3A6-5BFF-FD9A-DA13-7B7A2C23CCB3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>139699</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>111760</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C875FED5-9D4B-1B6A-6BDD-406B16CE2B6A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1664,14 +2860,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8210C0C-16A5-CD4D-8CBA-325C79473D67}">
-  <dimension ref="B2:G20"/>
+  <dimension ref="B2:I20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" customWidth="1"/>
     <col min="2" max="7" width="13.1640625" customWidth="1"/>
+    <col min="9" max="9" width="69.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -1684,252 +2881,256 @@
       <c r="E2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>5</v>
       </c>
+      <c r="I2" s="10" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="1">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B3" s="7">
         <v>90</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="7">
         <v>3</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="7">
         <v>0</v>
       </c>
       <c r="E3" s="2">
         <v>3.19</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="8">
         <f>AVERAGE(E3:E5)</f>
         <v>3.3166666666666664</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="4">
         <f>3/F3</f>
         <v>0.90452261306532666</v>
       </c>
+      <c r="I3" s="9" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
       <c r="E4" s="2">
         <v>3.39</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="I4" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
       <c r="E5" s="2">
         <v>3.37</v>
       </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7">
         <v>5</v>
       </c>
       <c r="E6" s="2">
         <v>3.84</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="8">
         <f t="shared" ref="F6" si="0">AVERAGE(E6:E8)</f>
         <v>3.9033333333333338</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="4">
         <f t="shared" ref="G6" si="1">3/F6</f>
         <v>0.76857386848847131</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
       <c r="E7" s="2">
         <v>3.83</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
       <c r="E8" s="2">
         <v>4.04</v>
       </c>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7">
         <v>10</v>
       </c>
       <c r="E9" s="2">
         <v>4.75</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="8">
         <f t="shared" ref="F9" si="2">AVERAGE(E9:E11)</f>
         <v>4.7733333333333334</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="4">
         <f t="shared" ref="G9" si="3">3/F9</f>
         <v>0.62849162011173187</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
       <c r="E10" s="2">
         <v>4.92</v>
       </c>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
       <c r="E11" s="2">
         <v>4.6500000000000004</v>
       </c>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7">
         <v>15</v>
       </c>
       <c r="E12" s="2">
         <v>7.31</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="8">
         <f t="shared" ref="F12" si="4">AVERAGE(E12:E14)</f>
         <v>7.4033333333333333</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="4">
         <f t="shared" ref="G12" si="5">3/F12</f>
         <v>0.40522287257991896</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
       <c r="E13" s="2">
         <v>7.48</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
       <c r="E14" s="2">
         <v>7.42</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1">
+    <row r="15" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7">
         <v>20</v>
       </c>
       <c r="E15" s="2">
         <v>8.98</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="8">
         <f t="shared" ref="F15" si="6">AVERAGE(E15:E17)</f>
         <v>8.6333333333333346</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="4">
         <f t="shared" ref="G15" si="7">3/F15</f>
         <v>0.34749034749034746</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
       <c r="E16" s="2">
         <v>8.51</v>
       </c>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
       <c r="E17" s="2">
         <v>8.41</v>
       </c>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1">
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7">
         <v>25</v>
       </c>
       <c r="E18" s="2">
         <v>12.5</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="8">
         <f t="shared" ref="F18" si="8">AVERAGE(E18:E20)</f>
         <v>12.106666666666667</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="4">
         <f t="shared" ref="G18" si="9">3/F18</f>
         <v>0.24779735682819382</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
       <c r="E19" s="2">
         <v>11.99</v>
       </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
       <c r="E20" s="2">
         <v>11.83</v>
       </c>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="G3:G5"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
     <mergeCell ref="G18:G20"/>
     <mergeCell ref="B3:B20"/>
     <mergeCell ref="C3:C20"/>
@@ -1945,6 +3146,11 @@
     <mergeCell ref="D12:D14"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="D18:D20"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -1952,4 +3158,161 @@
   </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FB1BF72-C9E0-F848-A1F8-3571E9B87CDF}">
+  <dimension ref="B2:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="2.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="7">
+        <v>250</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="D3" s="7">
+        <f>AVERAGE(C3:C5)</f>
+        <v>0.27666666666666667</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="7"/>
+      <c r="C4" s="1">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="12">
+        <f>((G3-0.0482)/0.001) + (G3*11)</f>
+        <v>962.8</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="7"/>
+      <c r="C5" s="1">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="D5" s="7"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="7">
+        <v>500</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D6" s="7">
+        <f t="shared" ref="D6" si="0">AVERAGE(C6:C8)</f>
+        <v>0.54666666666666675</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="7"/>
+      <c r="C7" s="1">
+        <v>0.54</v>
+      </c>
+      <c r="D7" s="7"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="7"/>
+      <c r="C8" s="1">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="7">
+        <v>750</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.78</v>
+      </c>
+      <c r="D9" s="7">
+        <f t="shared" ref="D9" si="1">AVERAGE(C9:C11)</f>
+        <v>0.77833333333333332</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="7"/>
+      <c r="C10" s="1">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="7"/>
+      <c r="C11" s="1">
+        <v>0.77</v>
+      </c>
+      <c r="D11" s="7"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="7">
+        <v>1000</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="7">
+        <f t="shared" ref="D12" si="2">AVERAGE(C12:C14)</f>
+        <v>1.0033333333333332</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="7"/>
+      <c r="C13" s="1">
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="7"/>
+      <c r="C14" s="1">
+        <v>1.0049999999999999</v>
+      </c>
+      <c r="D14" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B12:B14"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
benchmark 2 quad values calculation
</commit_message>
<xml_diff>
--- a/madi/301 speed data.xlsx
+++ b/madi/301 speed data.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madi/Desktop/COMPSYS301_team2/madi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6434248-AC0E-3649-BA0A-E8F6C8DA6138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A4A766-C6B4-B24C-BD14-8E8FC13D7710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" activeTab="1" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" activeTab="2" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
   </bookViews>
   <sheets>
     <sheet name="cmo speed" sheetId="1" r:id="rId1"/>
     <sheet name="quad encoder distance " sheetId="4" r:id="rId2"/>
+    <sheet name="benchmark speed quad values" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
   <si>
     <t>CMP Value</t>
   </si>
@@ -184,6 +185,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -193,22 +207,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1252,7 +1253,556 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
+              <a:endParaRPr lang="en-GB"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1248083968"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Distance</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> travelled vs quad encoder value</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="6.1681959176590521E-2"/>
+          <c:y val="2.9154507795769995E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'benchmark speed quad values'!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Avg Distance</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:forward val="100"/>
+            <c:backward val="100"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="3.9594097645962043E-2"/>
+                  <c:y val="-0.14594774934961496"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'benchmark speed quad values'!$B$3:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="3">
+                  <c:v>505</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1010</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'benchmark speed quad values'!$D$3:$D$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-5C52-2546-BCF6-B38F2F2963F8}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1248083968"/>
+        <c:axId val="1248096512"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1248083968"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Quad encoder value</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
               <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1248096512"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1248096512"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> travelled</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1429,6 +1979,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1946,6 +2536,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2527,6 +3633,49 @@
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>139699</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>111760</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3279AB6-7B38-DE4F-81A3-96E613050FB6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -2887,251 +4036,251 @@
       <c r="G2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>90</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>3</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="8">
         <v>0</v>
       </c>
       <c r="E3" s="2">
         <v>3.19</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="12">
         <f>AVERAGE(E3:E5)</f>
         <v>3.3166666666666664</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3" s="9">
         <f>3/F3</f>
         <v>0.90452261306532666</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
       <c r="E4" s="2">
         <v>3.39</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
       <c r="I4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
       <c r="E5" s="2">
         <v>3.37</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7">
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8">
         <v>5</v>
       </c>
       <c r="E6" s="2">
         <v>3.84</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="12">
         <f t="shared" ref="F6" si="0">AVERAGE(E6:E8)</f>
         <v>3.9033333333333338</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="9">
         <f t="shared" ref="G6" si="1">3/F6</f>
         <v>0.76857386848847131</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
       <c r="E7" s="2">
         <v>3.83</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
       <c r="E8" s="2">
         <v>4.04</v>
       </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7">
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8">
         <v>10</v>
       </c>
       <c r="E9" s="2">
         <v>4.75</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="12">
         <f t="shared" ref="F9" si="2">AVERAGE(E9:E11)</f>
         <v>4.7733333333333334</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="9">
         <f t="shared" ref="G9" si="3">3/F9</f>
         <v>0.62849162011173187</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
       <c r="E10" s="2">
         <v>4.92</v>
       </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="2">
         <v>4.6500000000000004</v>
       </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8">
         <v>15</v>
       </c>
       <c r="E12" s="2">
         <v>7.31</v>
       </c>
-      <c r="F12" s="8">
+      <c r="F12" s="12">
         <f t="shared" ref="F12" si="4">AVERAGE(E12:E14)</f>
         <v>7.4033333333333333</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="9">
         <f t="shared" ref="G12" si="5">3/F12</f>
         <v>0.40522287257991896</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
       <c r="E13" s="2">
         <v>7.48</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
       <c r="E14" s="2">
         <v>7.42</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8">
         <v>20</v>
       </c>
       <c r="E15" s="2">
         <v>8.98</v>
       </c>
-      <c r="F15" s="8">
+      <c r="F15" s="12">
         <f t="shared" ref="F15" si="6">AVERAGE(E15:E17)</f>
         <v>8.6333333333333346</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15" s="9">
         <f t="shared" ref="G15" si="7">3/F15</f>
         <v>0.34749034749034746</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
       <c r="E16" s="2">
         <v>8.51</v>
       </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
       <c r="E17" s="2">
         <v>8.41</v>
       </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8">
         <v>25</v>
       </c>
       <c r="E18" s="2">
         <v>12.5</v>
       </c>
-      <c r="F18" s="8">
+      <c r="F18" s="12">
         <f t="shared" ref="F18" si="8">AVERAGE(E18:E20)</f>
         <v>12.106666666666667</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="9">
         <f t="shared" ref="G18" si="9">3/F18</f>
         <v>0.24779735682819382</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
       <c r="E19" s="2">
         <v>11.99</v>
       </c>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
       <c r="E20" s="2">
         <v>11.83</v>
       </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G3:G5"/>
     <mergeCell ref="B3:B20"/>
     <mergeCell ref="C3:C20"/>
     <mergeCell ref="F3:F5"/>
@@ -3146,11 +4295,11 @@
     <mergeCell ref="D12:D14"/>
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="D18:D20"/>
-    <mergeCell ref="G3:G5"/>
     <mergeCell ref="G6:G8"/>
     <mergeCell ref="G9:G11"/>
     <mergeCell ref="G12:G14"/>
     <mergeCell ref="G15:G17"/>
+    <mergeCell ref="G18:G20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -3170,136 +4319,137 @@
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="15.5" customWidth="1"/>
     <col min="5" max="5" width="2.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>250</v>
       </c>
       <c r="C3" s="1">
         <v>0.28000000000000003</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="8">
         <f>AVERAGE(C3:C5)</f>
         <v>0.27666666666666667</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="12">
+        <v>2</v>
+      </c>
+      <c r="G3" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="7"/>
+      <c r="B4" s="8"/>
       <c r="C4" s="1">
         <v>0.27500000000000002</v>
       </c>
-      <c r="D4" s="7"/>
+      <c r="D4" s="8"/>
       <c r="F4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="7">
         <f>((G3-0.0482)/0.001) + (G3*11)</f>
         <v>962.8</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="7"/>
+      <c r="B5" s="8"/>
       <c r="C5" s="1">
         <v>0.27500000000000002</v>
       </c>
-      <c r="D5" s="7"/>
+      <c r="D5" s="8"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="7">
+      <c r="B6" s="8">
         <v>500</v>
       </c>
       <c r="C6" s="1">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="8">
         <f t="shared" ref="D6" si="0">AVERAGE(C6:C8)</f>
         <v>0.54666666666666675</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="7"/>
+      <c r="B7" s="8"/>
       <c r="C7" s="1">
         <v>0.54</v>
       </c>
-      <c r="D7" s="7"/>
+      <c r="D7" s="8"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="7"/>
+      <c r="B8" s="8"/>
       <c r="C8" s="1">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D8" s="7"/>
+      <c r="D8" s="8"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="7">
+      <c r="B9" s="8">
         <v>750</v>
       </c>
       <c r="C9" s="1">
         <v>0.78</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="8">
         <f t="shared" ref="D9" si="1">AVERAGE(C9:C11)</f>
         <v>0.77833333333333332</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B10" s="7"/>
+      <c r="B10" s="8"/>
       <c r="C10" s="1">
         <v>0.78500000000000003</v>
       </c>
-      <c r="D10" s="7"/>
+      <c r="D10" s="8"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B11" s="7"/>
+      <c r="B11" s="8"/>
       <c r="C11" s="1">
         <v>0.77</v>
       </c>
-      <c r="D11" s="7"/>
+      <c r="D11" s="8"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="7">
+      <c r="B12" s="8">
         <v>1000</v>
       </c>
       <c r="C12" s="1">
         <v>1</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="8">
         <f t="shared" ref="D12" si="2">AVERAGE(C12:C14)</f>
         <v>1.0033333333333332</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B13" s="7"/>
+      <c r="B13" s="8"/>
       <c r="C13" s="1">
         <v>1.0049999999999999</v>
       </c>
-      <c r="D13" s="7"/>
+      <c r="D13" s="8"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B14" s="7"/>
+      <c r="B14" s="8"/>
       <c r="C14" s="1">
         <v>1.0049999999999999</v>
       </c>
-      <c r="D14" s="7"/>
+      <c r="D14" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3315,4 +4465,146 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CF5B844-EAA3-3C44-B950-B2BC289A19FF}">
+  <dimension ref="B2:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15.5" customWidth="1"/>
+    <col min="5" max="5" width="2.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="8"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="8" t="e">
+        <f>AVERAGE(C3:C5)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="8"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="8"/>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="7">
+        <f>G3*1010</f>
+        <v>505</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="8"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="8"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="8">
+        <v>505</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="D6" s="8">
+        <f t="shared" ref="D6" si="0">AVERAGE(C6:C8)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="8"/>
+      <c r="C7" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="D7" s="8"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="8"/>
+      <c r="C8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="D8" s="8"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="8"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="8" t="e">
+        <f t="shared" ref="D9" si="1">AVERAGE(C9:C11)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="8"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="8"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="8"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="8"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="8">
+        <v>1010</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1</v>
+      </c>
+      <c r="D12" s="8">
+        <f t="shared" ref="D12" si="2">AVERAGE(C12:C14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="8"/>
+      <c r="C13" s="1">
+        <v>1</v>
+      </c>
+      <c r="D13" s="8"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="8"/>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+      <c r="D14" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="D9:D11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
speed data from benchmark test
</commit_message>
<xml_diff>
--- a/madi/301 speed data.xlsx
+++ b/madi/301 speed data.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/madi/Desktop/COMPSYS301_team2/madi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A4A766-C6B4-B24C-BD14-8E8FC13D7710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575C29E3-22E2-9745-96EF-40EC277BEA9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" activeTab="2" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
+    <workbookView xWindow="680" yWindow="660" windowWidth="28040" windowHeight="17160" activeTab="3" xr2:uid="{E44B5C4C-F08E-3F43-92EC-9F4C0D0CBAA3}"/>
   </bookViews>
   <sheets>
     <sheet name="cmo speed" sheetId="1" r:id="rId1"/>
     <sheet name="quad encoder distance " sheetId="4" r:id="rId2"/>
     <sheet name="benchmark speed quad values" sheetId="5" r:id="rId3"/>
+    <sheet name="30 september" sheetId="6" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
   <si>
     <t>CMP Value</t>
   </si>
@@ -81,6 +82,21 @@
   <si>
     <t>Quad</t>
   </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Average time</t>
+  </si>
+  <si>
+    <t>Speed</t>
+  </si>
+  <si>
+    <t>Compare value</t>
+  </si>
+  <si>
+    <t>Average speed</t>
+  </si>
 </sst>
 </file>
 
@@ -102,12 +118,54 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC6C6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7474"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC189F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6C3FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7CEB99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC5D3FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -174,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -208,6 +266,66 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1899,6 +2017,603 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Distance</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> vs quad encoder value</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'30 september'!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Avg Distance</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="38100" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:forward val="500"/>
+            <c:backward val="250"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:forward val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="0.14096631721636069"/>
+                  <c:y val="-0.3315342426441612"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'30 september'!$C$3:$C$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>600</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>900</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1800</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1439</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1550</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1661</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1328</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'30 september'!$E$3:$E$32</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="30"/>
+                <c:pt idx="0">
+                  <c:v>0.27166666666666667</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.53166666666666673</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.79333333333333333</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0449999999999999</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.3216666666666665</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1.5883333333333332</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.27</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1.3666666666666669</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>1.4683333333333335</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>1.171</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D4D1-9D43-8C15-3347DD31C914}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1147459711"/>
+        <c:axId val="1147466879"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1147459711"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Quad</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> encoder value</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147466879"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1147466879"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1147459711"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2019,6 +2734,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3052,6 +3807,522 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3676,6 +4947,47 @@
         <xdr:cNvGraphicFramePr>
           <a:graphicFrameLocks/>
         </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>128863</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>68156</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>31093</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>167024</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A05CD0D-BC69-2692-4392-9570D612F968}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -4280,6 +5592,10 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="G18:G20"/>
     <mergeCell ref="G3:G5"/>
     <mergeCell ref="B3:B20"/>
     <mergeCell ref="C3:C20"/>
@@ -4296,10 +5612,6 @@
     <mergeCell ref="D15:D17"/>
     <mergeCell ref="D18:D20"/>
     <mergeCell ref="G6:G8"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="G18:G20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -4607,4 +5919,605 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0627EEC0-B386-684E-9E68-3B0CFE0ABCEC}">
+  <dimension ref="B2:K32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3.6640625" style="15" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" style="15" customWidth="1"/>
+    <col min="3" max="3" width="17.5" style="15" customWidth="1"/>
+    <col min="4" max="4" width="15" style="15" customWidth="1"/>
+    <col min="5" max="8" width="15.5" style="15" customWidth="1"/>
+    <col min="9" max="9" width="2.83203125" style="15" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" style="15" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="15" customWidth="1"/>
+    <col min="12" max="16384" width="10.83203125" style="15"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B3" s="9">
+        <v>20</v>
+      </c>
+      <c r="C3" s="22">
+        <v>300</v>
+      </c>
+      <c r="D3" s="23">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="E3" s="22">
+        <f>AVERAGE(D3:D5)</f>
+        <v>0.27166666666666667</v>
+      </c>
+      <c r="F3" s="23">
+        <v>1.06</v>
+      </c>
+      <c r="G3" s="24">
+        <f>AVERAGE(F3:F5)</f>
+        <v>1.0999999999999999</v>
+      </c>
+      <c r="H3" s="24">
+        <f>E3/G3</f>
+        <v>0.24696969696969701</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="K3" s="16">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B4" s="10"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23">
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="E4" s="22"/>
+      <c r="F4" s="23">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="J4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="16">
+        <f>(K3-0.0034)/0.0009 + 50</f>
+        <v>1601.7777777777776</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="10"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="23">
+        <v>0.26500000000000001</v>
+      </c>
+      <c r="E5" s="22"/>
+      <c r="F5" s="23">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="G5" s="26"/>
+      <c r="H5" s="26"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="10"/>
+      <c r="C6" s="22">
+        <v>600</v>
+      </c>
+      <c r="D6" s="23">
+        <v>0.53500000000000003</v>
+      </c>
+      <c r="E6" s="22">
+        <f t="shared" ref="E6" si="0">AVERAGE(D6:D8)</f>
+        <v>0.53166666666666673</v>
+      </c>
+      <c r="F6" s="23">
+        <v>2.16</v>
+      </c>
+      <c r="G6" s="24">
+        <f t="shared" ref="G6" si="1">AVERAGE(F6:F8)</f>
+        <v>2.0866666666666669</v>
+      </c>
+      <c r="H6" s="24">
+        <f t="shared" ref="H6" si="2">E6/G6</f>
+        <v>0.25479233226837061</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="17">
+        <f>AVERAGE(H3:H20,H24:H32)</f>
+        <v>0.26018951225190562</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B7" s="10"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="23">
+        <v>0.52</v>
+      </c>
+      <c r="E7" s="22"/>
+      <c r="F7" s="23">
+        <v>2.06</v>
+      </c>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="10"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="23">
+        <v>0.54</v>
+      </c>
+      <c r="E8" s="22"/>
+      <c r="F8" s="23">
+        <v>2.04</v>
+      </c>
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="10"/>
+      <c r="C9" s="22">
+        <v>900</v>
+      </c>
+      <c r="D9" s="23">
+        <v>0.8</v>
+      </c>
+      <c r="E9" s="22">
+        <f t="shared" ref="E9" si="3">AVERAGE(D9:D11)</f>
+        <v>0.79333333333333333</v>
+      </c>
+      <c r="F9" s="23">
+        <v>3.13</v>
+      </c>
+      <c r="G9" s="24">
+        <f t="shared" ref="G9" si="4">AVERAGE(F9:F11)</f>
+        <v>3.27</v>
+      </c>
+      <c r="H9" s="24">
+        <f t="shared" ref="H9" si="5">E9/G9</f>
+        <v>0.24260958205912334</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="10"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23">
+        <v>0.79</v>
+      </c>
+      <c r="E10" s="22"/>
+      <c r="F10" s="23">
+        <v>3.21</v>
+      </c>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="10"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="23">
+        <v>0.79</v>
+      </c>
+      <c r="E11" s="22"/>
+      <c r="F11" s="23">
+        <v>3.47</v>
+      </c>
+      <c r="G11" s="26"/>
+      <c r="H11" s="26"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B12" s="10"/>
+      <c r="C12" s="22">
+        <v>1200</v>
+      </c>
+      <c r="D12" s="23">
+        <v>1.0349999999999999</v>
+      </c>
+      <c r="E12" s="22">
+        <f>AVERAGE(D12:D14)</f>
+        <v>1.0449999999999999</v>
+      </c>
+      <c r="F12" s="23">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="G12" s="24">
+        <f>AVERAGE(F12:F14)</f>
+        <v>4.1099999999999994</v>
+      </c>
+      <c r="H12" s="24">
+        <f t="shared" ref="H12" si="6">E12/G12</f>
+        <v>0.2542579075425791</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B13" s="10"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23">
+        <v>1.0449999999999999</v>
+      </c>
+      <c r="E13" s="22"/>
+      <c r="F13" s="23">
+        <v>4.05</v>
+      </c>
+      <c r="G13" s="25"/>
+      <c r="H13" s="25"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B14" s="10"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="23">
+        <v>1.0549999999999999</v>
+      </c>
+      <c r="E14" s="22"/>
+      <c r="F14" s="23">
+        <v>4.13</v>
+      </c>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B15" s="10"/>
+      <c r="C15" s="24">
+        <v>1500</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1.325</v>
+      </c>
+      <c r="E15" s="22">
+        <f t="shared" ref="E15" si="7">AVERAGE(D15:D17)</f>
+        <v>1.3216666666666665</v>
+      </c>
+      <c r="F15" s="23">
+        <v>4.97</v>
+      </c>
+      <c r="G15" s="24">
+        <f t="shared" ref="G15" si="8">AVERAGE(F15:F17)</f>
+        <v>5.0299999999999994</v>
+      </c>
+      <c r="H15" s="24">
+        <f t="shared" ref="H15:H18" si="9">E15/G15</f>
+        <v>0.26275679257786616</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B16" s="10"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="23">
+        <v>1.32</v>
+      </c>
+      <c r="E16" s="22"/>
+      <c r="F16" s="23">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B17" s="10"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="23">
+        <v>1.32</v>
+      </c>
+      <c r="E17" s="22"/>
+      <c r="F17" s="23">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B18" s="10"/>
+      <c r="C18" s="24">
+        <v>1800</v>
+      </c>
+      <c r="D18" s="23">
+        <v>1.585</v>
+      </c>
+      <c r="E18" s="22">
+        <f t="shared" ref="E18" si="10">AVERAGE(D18:D20)</f>
+        <v>1.5883333333333332</v>
+      </c>
+      <c r="F18" s="23">
+        <v>5.91</v>
+      </c>
+      <c r="G18" s="24">
+        <f t="shared" ref="G18" si="11">AVERAGE(F18:F20)</f>
+        <v>5.9200000000000008</v>
+      </c>
+      <c r="H18" s="24">
+        <f t="shared" si="9"/>
+        <v>0.26829954954954949</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B19" s="10"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="23">
+        <v>1.585</v>
+      </c>
+      <c r="E19" s="22"/>
+      <c r="F19" s="23">
+        <v>5.9</v>
+      </c>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" s="10"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="23">
+        <v>1.595</v>
+      </c>
+      <c r="E20" s="22"/>
+      <c r="F20" s="23">
+        <v>5.95</v>
+      </c>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21" s="10"/>
+      <c r="C21" s="27">
+        <v>1439</v>
+      </c>
+      <c r="D21" s="28">
+        <v>1.2649999999999999</v>
+      </c>
+      <c r="E21" s="27">
+        <f t="shared" ref="E21" si="12">AVERAGE(D21:D23)</f>
+        <v>1.27</v>
+      </c>
+      <c r="F21" s="18"/>
+      <c r="G21" s="19"/>
+      <c r="H21" s="19" t="e">
+        <f t="shared" ref="H21:H27" si="13">E21/G21</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B22" s="10"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="28">
+        <v>1.27</v>
+      </c>
+      <c r="E22" s="27"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B23" s="10"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="28">
+        <v>1.2749999999999999</v>
+      </c>
+      <c r="E23" s="27"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B24" s="10"/>
+      <c r="C24" s="29">
+        <v>1550</v>
+      </c>
+      <c r="D24" s="28">
+        <v>1.365</v>
+      </c>
+      <c r="E24" s="27">
+        <f t="shared" ref="E24" si="14">AVERAGE(D24:D26)</f>
+        <v>1.3666666666666669</v>
+      </c>
+      <c r="F24" s="28">
+        <v>4.97</v>
+      </c>
+      <c r="G24" s="29">
+        <f t="shared" ref="G21:G24" si="15">AVERAGE(F24:F26)</f>
+        <v>5.0766666666666671</v>
+      </c>
+      <c r="H24" s="29">
+        <f t="shared" si="13"/>
+        <v>0.26920551543007226</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B25" s="10"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="28">
+        <v>1.37</v>
+      </c>
+      <c r="E25" s="27"/>
+      <c r="F25" s="28">
+        <v>5.13</v>
+      </c>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B26" s="10"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="28">
+        <v>1.365</v>
+      </c>
+      <c r="E26" s="27"/>
+      <c r="F26" s="28">
+        <v>5.13</v>
+      </c>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B27" s="10"/>
+      <c r="C27" s="29">
+        <v>1661</v>
+      </c>
+      <c r="D27" s="28">
+        <v>1.47</v>
+      </c>
+      <c r="E27" s="27">
+        <f t="shared" ref="E27" si="16">AVERAGE(D27:D29)</f>
+        <v>1.4683333333333335</v>
+      </c>
+      <c r="F27" s="28">
+        <v>5.5</v>
+      </c>
+      <c r="G27" s="29">
+        <f t="shared" ref="G27" si="17">AVERAGE(F27:F29)</f>
+        <v>5.4200000000000008</v>
+      </c>
+      <c r="H27" s="29">
+        <f t="shared" si="13"/>
+        <v>0.27091020910209102</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B28" s="10"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="32">
+        <v>1.4750000000000001</v>
+      </c>
+      <c r="E28" s="27"/>
+      <c r="F28" s="28">
+        <v>5.4</v>
+      </c>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B29" s="10"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="28">
+        <v>1.46</v>
+      </c>
+      <c r="E29" s="27"/>
+      <c r="F29" s="28">
+        <v>5.36</v>
+      </c>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B30" s="10"/>
+      <c r="C30" s="29">
+        <v>1328</v>
+      </c>
+      <c r="D30" s="28">
+        <v>1.17</v>
+      </c>
+      <c r="E30" s="27">
+        <f t="shared" ref="E30" si="18">AVERAGE(D30:D32)</f>
+        <v>1.171</v>
+      </c>
+      <c r="F30" s="28">
+        <v>4.32</v>
+      </c>
+      <c r="G30" s="29">
+        <f t="shared" ref="G30" si="19">AVERAGE(F30:F32)</f>
+        <v>4.3066666666666666</v>
+      </c>
+      <c r="H30" s="29">
+        <f t="shared" ref="H30" si="20">E30/G30</f>
+        <v>0.27190402476780184</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B31" s="10"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="28">
+        <v>1.18</v>
+      </c>
+      <c r="E31" s="27"/>
+      <c r="F31" s="28">
+        <v>4.2699999999999996</v>
+      </c>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B32" s="11"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="28">
+        <v>1.163</v>
+      </c>
+      <c r="E32" s="27"/>
+      <c r="F32" s="28">
+        <v>4.33</v>
+      </c>
+      <c r="G32" s="31"/>
+      <c r="H32" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="C30:C32"/>
+    <mergeCell ref="E30:E32"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="B3:B32"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="E24:E26"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="H18:H20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="H6:H8"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="C9:C11"/>
+    <mergeCell ref="E9:E11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>